<commit_message>
Revert shoulder press to seated dumbbell (Smith machine too low for 188cm)
Standing Smith machine press hits ceiling at full extension for a 188cm user. Swapped back to seated dumbbell shoulder press across all DI sheets, technique sheet, and dashboard.

https://claude.ai/code/session_01GVJ1XP4t8b95djSt71eE5q
</commit_message>
<xml_diff>
--- a/fitness_plan_david_v4.xlsx
+++ b/fitness_plan_david_v4.xlsx
@@ -825,7 +825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:K42"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1098,11 +1098,19 @@
           <t>Klimmzüge (Pull-Up Bar)</t>
         </is>
       </c>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="7" t="n"/>
       <c r="E15" s="15" t="inlineStr">
         <is>
           <t>Solo trainierbar — echte Lats-Übung statt nur Kabel</t>
         </is>
       </c>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="10" t="n"/>
+      <c r="H15" s="10" t="n"/>
+      <c r="I15" s="10" t="n"/>
+      <c r="J15" s="10" t="n"/>
+      <c r="K15" s="7" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="B16" s="14" t="inlineStr">
@@ -1110,11 +1118,19 @@
           <t>Freie Kniebeugen (Rack)</t>
         </is>
       </c>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="7" t="n"/>
       <c r="E16" s="16" t="inlineStr">
         <is>
           <t>Aus J-Hooks — endlich echte Langhantel-Squats möglich</t>
         </is>
       </c>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="10" t="n"/>
+      <c r="H16" s="10" t="n"/>
+      <c r="I16" s="10" t="n"/>
+      <c r="J16" s="10" t="n"/>
+      <c r="K16" s="7" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="B17" s="14" t="inlineStr">
@@ -1122,11 +1138,19 @@
           <t>Smith Machine Presses</t>
         </is>
       </c>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="7" t="n"/>
       <c r="E17" s="15" t="inlineStr">
         <is>
           <t>Solo sicher — kein Spotter nötig, fixierte Bahn = mehr Fokus</t>
         </is>
       </c>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="10" t="n"/>
+      <c r="H17" s="10" t="n"/>
+      <c r="I17" s="10" t="n"/>
+      <c r="J17" s="10" t="n"/>
+      <c r="K17" s="7" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="B18" s="14" t="inlineStr">
@@ -1134,11 +1158,19 @@
           <t>Rack Pulls / RDL aus J-Hooks</t>
         </is>
       </c>
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="7" t="n"/>
       <c r="E18" s="16" t="inlineStr">
         <is>
           <t>Kein Boden-Lift nötig — schont unteren Rücken beim Aufwärmen</t>
         </is>
       </c>
+      <c r="F18" s="10" t="n"/>
+      <c r="G18" s="10" t="n"/>
+      <c r="H18" s="10" t="n"/>
+      <c r="I18" s="10" t="n"/>
+      <c r="J18" s="10" t="n"/>
+      <c r="K18" s="7" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="B19" s="14" t="inlineStr">
@@ -1146,12 +1178,21 @@
           <t>Bulgarian Split Squat Smith</t>
         </is>
       </c>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="7" t="n"/>
       <c r="E19" s="15" t="inlineStr">
         <is>
           <t>Stabiler als frei — mehr Gewicht sicher möglich</t>
         </is>
       </c>
-    </row>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="10" t="n"/>
+      <c r="H19" s="10" t="n"/>
+      <c r="I19" s="10" t="n"/>
+      <c r="J19" s="10" t="n"/>
+      <c r="K19" s="7" t="n"/>
+    </row>
+    <row r="20"/>
     <row r="21" ht="12" customHeight="1"/>
     <row r="22" ht="26" customHeight="1">
       <c r="B22" s="3" t="inlineStr">
@@ -1251,11 +1292,11 @@
     <row r="26" ht="20" customHeight="1">
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Schulterdrücken Smith Machine</t>
+          <t>Schulterdrücken KH sitzend</t>
         </is>
       </c>
       <c r="C26" s="17" t="n">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="D26" s="18" t="n"/>
       <c r="E26" s="18" t="n"/>
@@ -2377,6 +2418,8 @@
         </is>
       </c>
       <c r="J23" s="47" t="n"/>
+      <c r="K23" s="10" t="n"/>
+      <c r="L23" s="7" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="B25" s="31" t="inlineStr">
@@ -2838,7 +2881,7 @@
       </c>
       <c r="C14" s="36" t="inlineStr">
         <is>
-          <t>Schulterdrücken Smith Machine stehend</t>
+          <t>Schulterdrücken KH sitzend</t>
         </is>
       </c>
       <c r="D14" s="37" t="inlineStr">
@@ -2847,7 +2890,7 @@
         </is>
       </c>
       <c r="E14" s="38" t="n">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="F14" s="39" t="inlineStr">
         <is>
@@ -2857,7 +2900,7 @@
       <c r="G14" s="18" t="inlineStr"/>
       <c r="H14" s="18" t="inlineStr"/>
       <c r="I14" s="38" t="n">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="J14" s="39" t="inlineStr">
         <is>
@@ -2867,7 +2910,7 @@
       <c r="K14" s="18" t="inlineStr"/>
       <c r="L14" s="18" t="inlineStr"/>
       <c r="M14" s="38" t="n">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="N14" s="39" t="inlineStr">
         <is>
@@ -2877,7 +2920,7 @@
       <c r="O14" s="18" t="inlineStr"/>
       <c r="P14" s="18" t="inlineStr"/>
       <c r="Q14" s="38" t="n">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="R14" s="39" t="inlineStr">
         <is>
@@ -2888,7 +2931,7 @@
       <c r="T14" s="18" t="inlineStr"/>
       <c r="U14" s="40" t="inlineStr">
         <is>
-          <t>Smith = stabiler als frei, mehr Gewicht möglich</t>
+          <t>Smith Machine zu niedrig (188cm) — KH frei, kein Deckenkontakt</t>
         </is>
       </c>
     </row>
@@ -3122,6 +3165,8 @@
         </is>
       </c>
       <c r="J21" s="47" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="31" t="inlineStr">
@@ -3869,6 +3914,8 @@
         </is>
       </c>
       <c r="J21" s="47" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="31" t="inlineStr">
@@ -4602,6 +4649,8 @@
         </is>
       </c>
       <c r="J21" s="47" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="51" t="inlineStr">
@@ -5443,6 +5492,8 @@
         </is>
       </c>
       <c r="J23" s="47" t="n"/>
+      <c r="K23" s="10" t="n"/>
+      <c r="L23" s="7" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="B25" s="31" t="inlineStr">
@@ -5904,7 +5955,7 @@
       </c>
       <c r="C14" s="36" t="inlineStr">
         <is>
-          <t>Schulterdrücken Smith Machine stehend</t>
+          <t>Schulterdrücken KH sitzend</t>
         </is>
       </c>
       <c r="D14" s="37" t="inlineStr">
@@ -5913,7 +5964,7 @@
         </is>
       </c>
       <c r="E14" s="38" t="n">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="F14" s="39" t="inlineStr">
         <is>
@@ -5923,7 +5974,7 @@
       <c r="G14" s="18" t="inlineStr"/>
       <c r="H14" s="18" t="inlineStr"/>
       <c r="I14" s="38" t="n">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="J14" s="39" t="inlineStr">
         <is>
@@ -5933,7 +5984,7 @@
       <c r="K14" s="18" t="inlineStr"/>
       <c r="L14" s="18" t="inlineStr"/>
       <c r="M14" s="38" t="n">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="N14" s="39" t="inlineStr">
         <is>
@@ -5943,7 +5994,7 @@
       <c r="O14" s="18" t="inlineStr"/>
       <c r="P14" s="18" t="inlineStr"/>
       <c r="Q14" s="38" t="n">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="R14" s="39" t="inlineStr">
         <is>
@@ -5954,7 +6005,7 @@
       <c r="T14" s="18" t="inlineStr"/>
       <c r="U14" s="40" t="inlineStr">
         <is>
-          <t>Smith = stabiler als frei, mehr Gewicht möglich</t>
+          <t>Smith Machine zu niedrig (188cm) — KH frei, kein Deckenkontakt</t>
         </is>
       </c>
     </row>
@@ -6188,6 +6239,8 @@
         </is>
       </c>
       <c r="J21" s="47" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="31" t="inlineStr">
@@ -6935,6 +6988,8 @@
         </is>
       </c>
       <c r="J21" s="47" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="31" t="inlineStr">
@@ -7668,6 +7723,8 @@
         </is>
       </c>
       <c r="J21" s="47" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="51" t="inlineStr">
@@ -8509,6 +8566,8 @@
         </is>
       </c>
       <c r="J23" s="47" t="n"/>
+      <c r="K23" s="10" t="n"/>
+      <c r="L23" s="7" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="B25" s="31" t="inlineStr">
@@ -8548,7 +8607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E34"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -8662,7 +8721,7 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Schulterdrücken Smith Machine stehend</t>
+          <t>Schulterdrücken KH sitzend</t>
         </is>
       </c>
       <c r="D8" s="26" t="inlineStr">
@@ -8672,7 +8731,7 @@
       </c>
       <c r="E8" s="25" t="inlineStr">
         <is>
-          <t>▶  YouTube Tutorial öffnen →  Schulterdrücken Smith Machine stehend</t>
+          <t>▶  YouTube Tutorial öffnen →  Schulterdrücken KH sitzend</t>
         </is>
       </c>
     </row>
@@ -9665,7 +9724,7 @@
       </c>
       <c r="C14" s="36" t="inlineStr">
         <is>
-          <t>Schulterdrücken Smith Machine stehend</t>
+          <t>Schulterdrücken KH sitzend</t>
         </is>
       </c>
       <c r="D14" s="37" t="inlineStr">
@@ -9674,7 +9733,7 @@
         </is>
       </c>
       <c r="E14" s="38" t="n">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="F14" s="39" t="inlineStr">
         <is>
@@ -9684,7 +9743,7 @@
       <c r="G14" s="18" t="inlineStr"/>
       <c r="H14" s="18" t="inlineStr"/>
       <c r="I14" s="38" t="n">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="J14" s="39" t="inlineStr">
         <is>
@@ -9694,7 +9753,7 @@
       <c r="K14" s="18" t="inlineStr"/>
       <c r="L14" s="18" t="inlineStr"/>
       <c r="M14" s="38" t="n">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="N14" s="39" t="inlineStr">
         <is>
@@ -9704,7 +9763,7 @@
       <c r="O14" s="18" t="inlineStr"/>
       <c r="P14" s="18" t="inlineStr"/>
       <c r="Q14" s="38" t="n">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="R14" s="39" t="inlineStr">
         <is>
@@ -9715,7 +9774,7 @@
       <c r="T14" s="18" t="inlineStr"/>
       <c r="U14" s="40" t="inlineStr">
         <is>
-          <t>Smith = stabiler als frei, mehr Gewicht möglich</t>
+          <t>Smith Machine zu niedrig (188cm) — KH frei, kein Deckenkontakt</t>
         </is>
       </c>
     </row>
@@ -9949,6 +10008,8 @@
         </is>
       </c>
       <c r="J21" s="47" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="31" t="inlineStr">
@@ -10696,6 +10757,8 @@
         </is>
       </c>
       <c r="J21" s="47" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="31" t="inlineStr">
@@ -11429,6 +11492,8 @@
         </is>
       </c>
       <c r="J21" s="47" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="51" t="inlineStr">
@@ -12270,6 +12335,8 @@
         </is>
       </c>
       <c r="J23" s="47" t="n"/>
+      <c r="K23" s="10" t="n"/>
+      <c r="L23" s="7" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="B25" s="31" t="inlineStr">
@@ -12731,7 +12798,7 @@
       </c>
       <c r="C14" s="36" t="inlineStr">
         <is>
-          <t>Schulterdrücken Smith Machine stehend</t>
+          <t>Schulterdrücken KH sitzend</t>
         </is>
       </c>
       <c r="D14" s="37" t="inlineStr">
@@ -12740,7 +12807,7 @@
         </is>
       </c>
       <c r="E14" s="38" t="n">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="F14" s="39" t="inlineStr">
         <is>
@@ -12750,7 +12817,7 @@
       <c r="G14" s="18" t="inlineStr"/>
       <c r="H14" s="18" t="inlineStr"/>
       <c r="I14" s="38" t="n">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="J14" s="39" t="inlineStr">
         <is>
@@ -12760,7 +12827,7 @@
       <c r="K14" s="18" t="inlineStr"/>
       <c r="L14" s="18" t="inlineStr"/>
       <c r="M14" s="38" t="n">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="N14" s="39" t="inlineStr">
         <is>
@@ -12770,7 +12837,7 @@
       <c r="O14" s="18" t="inlineStr"/>
       <c r="P14" s="18" t="inlineStr"/>
       <c r="Q14" s="38" t="n">
-        <v>20</v>
+        <v>17.5</v>
       </c>
       <c r="R14" s="39" t="inlineStr">
         <is>
@@ -12781,7 +12848,7 @@
       <c r="T14" s="18" t="inlineStr"/>
       <c r="U14" s="40" t="inlineStr">
         <is>
-          <t>Smith = stabiler als frei, mehr Gewicht möglich</t>
+          <t>Smith Machine zu niedrig (188cm) — KH frei, kein Deckenkontakt</t>
         </is>
       </c>
     </row>
@@ -13015,6 +13082,8 @@
         </is>
       </c>
       <c r="J21" s="47" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="31" t="inlineStr">
@@ -13762,6 +13831,8 @@
         </is>
       </c>
       <c r="J21" s="47" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="31" t="inlineStr">
@@ -14495,6 +14566,8 @@
         </is>
       </c>
       <c r="J21" s="47" t="n"/>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="51" t="inlineStr">

</xml_diff>

<commit_message>
Set incline bench angle to 40 degrees (closest available to optimal 30-45 range)
User's bench only supports 0/20/40/55/85 degrees. 40 is the best fit for upper chest EMG activation.

https://claude.ai/code/session_01GVJ1XP4t8b95djSt71eE5q
</commit_message>
<xml_diff>
--- a/fitness_plan_david_v4.xlsx
+++ b/fitness_plan_david_v4.xlsx
@@ -825,7 +825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K42"/>
+  <dimension ref="B2:K42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1192,7 +1192,6 @@
       <c r="J19" s="10" t="n"/>
       <c r="K19" s="7" t="n"/>
     </row>
-    <row r="20"/>
     <row r="21" ht="12" customHeight="1"/>
     <row r="22" ht="26" customHeight="1">
       <c r="B22" s="3" t="inlineStr">
@@ -2459,7 +2458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:V23"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2684,7 +2683,7 @@
       </c>
       <c r="C9" s="36" t="inlineStr">
         <is>
-          <t>Schrägbank Drücken Smith Machine (30°)</t>
+          <t>Schrägbank Drücken Smith Machine (40°)</t>
         </is>
       </c>
       <c r="D9" s="37" t="inlineStr">
@@ -2734,7 +2733,7 @@
       <c r="T9" s="18" t="inlineStr"/>
       <c r="U9" s="40" t="inlineStr">
         <is>
-          <t>Fixierte Bahn = konstanter Winkel, sicher solo</t>
+          <t>40° = beste Oberbrust-Aktivierung bei deiner Bank</t>
         </is>
       </c>
     </row>
@@ -3168,6 +3167,7 @@
       <c r="K21" s="10" t="n"/>
       <c r="L21" s="7" t="n"/>
     </row>
+    <row r="22"/>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="31" t="inlineStr">
         <is>
@@ -5533,7 +5533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:V23"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -5758,7 +5758,7 @@
       </c>
       <c r="C9" s="36" t="inlineStr">
         <is>
-          <t>Schrägbank Drücken Smith Machine (30°)</t>
+          <t>Schrägbank Drücken Smith Machine (40°)</t>
         </is>
       </c>
       <c r="D9" s="37" t="inlineStr">
@@ -5808,7 +5808,7 @@
       <c r="T9" s="18" t="inlineStr"/>
       <c r="U9" s="40" t="inlineStr">
         <is>
-          <t>Fixierte Bahn = konstanter Winkel, sicher solo</t>
+          <t>40° = beste Oberbrust-Aktivierung bei deiner Bank</t>
         </is>
       </c>
     </row>
@@ -6242,6 +6242,7 @@
       <c r="K21" s="10" t="n"/>
       <c r="L21" s="7" t="n"/>
     </row>
+    <row r="22"/>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="31" t="inlineStr">
         <is>
@@ -8661,7 +8662,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Schrägbank Drücken Smith Machine (30°)</t>
+          <t>Schrägbank Drücken Smith Machine (40°)</t>
         </is>
       </c>
       <c r="D5" s="24" t="inlineStr">
@@ -9302,7 +9303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:V23"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -9527,7 +9528,7 @@
       </c>
       <c r="C9" s="36" t="inlineStr">
         <is>
-          <t>Schrägbank Drücken Smith Machine (30°)</t>
+          <t>Schrägbank Drücken Smith Machine (40°)</t>
         </is>
       </c>
       <c r="D9" s="37" t="inlineStr">
@@ -9577,7 +9578,7 @@
       <c r="T9" s="18" t="inlineStr"/>
       <c r="U9" s="40" t="inlineStr">
         <is>
-          <t>Fixierte Bahn = konstanter Winkel, sicher solo</t>
+          <t>40° = beste Oberbrust-Aktivierung bei deiner Bank</t>
         </is>
       </c>
     </row>
@@ -10011,6 +10012,7 @@
       <c r="K21" s="10" t="n"/>
       <c r="L21" s="7" t="n"/>
     </row>
+    <row r="22"/>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="31" t="inlineStr">
         <is>
@@ -12376,7 +12378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:V23"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -12601,7 +12603,7 @@
       </c>
       <c r="C9" s="36" t="inlineStr">
         <is>
-          <t>Schrägbank Drücken Smith Machine (30°)</t>
+          <t>Schrägbank Drücken Smith Machine (40°)</t>
         </is>
       </c>
       <c r="D9" s="37" t="inlineStr">
@@ -12651,7 +12653,7 @@
       <c r="T9" s="18" t="inlineStr"/>
       <c r="U9" s="40" t="inlineStr">
         <is>
-          <t>Fixierte Bahn = konstanter Winkel, sicher solo</t>
+          <t>40° = beste Oberbrust-Aktivierung bei deiner Bank</t>
         </is>
       </c>
     </row>
@@ -13085,6 +13087,7 @@
       <c r="K21" s="10" t="n"/>
       <c r="L21" s="7" t="n"/>
     </row>
+    <row r="22"/>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="31" t="inlineStr">
         <is>

</xml_diff>